<commit_message>
Commit final du 22/06/2026
</commit_message>
<xml_diff>
--- a/PM_Fontenay sous bois.xlsx
+++ b/PM_Fontenay sous bois.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F73"/>
+  <dimension ref="A1:F87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2075,12 +2075,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Fontenay-sous-Bois Principal</t>
+          <t>Pharmacie Bellenger</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>poste</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -2089,26 +2089,26 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>48.8490985</v>
+        <v>48.8529337</v>
       </c>
       <c r="E60" t="n">
-        <v>2.4755055</v>
+        <v>2.4572463</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>48.8490985, 2.4755055</t>
+          <t>48.8529337, 2.4572463</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Fontenay-sous-Bois Rigollots</t>
+          <t>Pharmacie Bertrand</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>poste</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2117,26 +2117,26 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>48.848805</v>
+        <v>48.8515568</v>
       </c>
       <c r="E61" t="n">
-        <v>2.4579266</v>
+        <v>2.4763174</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>48.848805, 2.4579266</t>
+          <t>48.8515568, 2.4763174</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Relais Postal</t>
+          <t>Pharmacie Betty Taieb</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>poste</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2145,26 +2145,26 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>48.853931</v>
+        <v>48.8527636</v>
       </c>
       <c r="E62" t="n">
-        <v>2.4695139</v>
+        <v>2.4569447</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>48.853931, 2.4695139</t>
+          <t>48.8527636, 2.4569447</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Val-de-Fontenay</t>
+          <t>Pharmacie Dalayrac</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>poste</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2173,26 +2173,26 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>48.853767</v>
+        <v>48.8493082</v>
       </c>
       <c r="E63" t="n">
-        <v>2.4876008</v>
+        <v>2.4576252</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>48.853767, 2.4876008</t>
+          <t>48.8493082, 2.4576252</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Auchan</t>
+          <t>Pharmacie Fraysse RER</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>supermarché</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2201,26 +2201,26 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>48.8532361</v>
+        <v>48.8438943</v>
       </c>
       <c r="E64" t="n">
-        <v>2.4827546</v>
+        <v>2.4662063</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>48.8532361, 2.4827546</t>
+          <t>48.8438943, 2.4662063</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Diagonal</t>
+          <t>Pharmacie Godkine</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>supermarché</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -2229,26 +2229,26 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>48.8559879</v>
+        <v>48.8559629</v>
       </c>
       <c r="E65" t="n">
-        <v>2.4784523</v>
+        <v>2.482184</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>48.8559879, 2.4784523</t>
+          <t>48.8559629, 2.482184</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Hyper Casher</t>
+          <t>Pharmacie Khiat</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>supermarché</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -2257,26 +2257,26 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>48.8546063</v>
+        <v>48.8497894</v>
       </c>
       <c r="E66" t="n">
-        <v>2.4689527</v>
+        <v>2.4562925</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>48.8546063, 2.4689527</t>
+          <t>48.8497894, 2.4562925</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Intermarché</t>
+          <t>Pharmacie Saint-Germain</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>supermarché</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2285,26 +2285,26 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>48.8495365</v>
+        <v>48.8466291</v>
       </c>
       <c r="E67" t="n">
-        <v>2.48986</v>
+        <v>2.4708282</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>48.8495365, 2.48986</t>
+          <t>48.8466291, 2.4708282</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Lidl</t>
+          <t>Pharmacie Talamoni</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>supermarché</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2313,26 +2313,26 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>48.8485331</v>
+        <v>48.857733</v>
       </c>
       <c r="E68" t="n">
-        <v>2.4886907</v>
+        <v>2.4712005</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>48.8485331, 2.4886907</t>
+          <t>48.857733, 2.4712005</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Monoprix</t>
+          <t>Pharmacie Val de Fontenay</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>supermarché</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -2341,26 +2341,26 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>48.8493017</v>
+        <v>48.8537108</v>
       </c>
       <c r="E69" t="n">
-        <v>2.458854</v>
+        <v>2.4843578</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>48.8493017, 2.458854</t>
+          <t>48.8537108, 2.4843578</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Naturalia</t>
+          <t>Pharmacie des Arts</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>supermarché</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -2369,26 +2369,26 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>48.8486498</v>
+        <v>48.8520934</v>
       </c>
       <c r="E70" t="n">
-        <v>2.459837</v>
+        <v>2.4849953</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>48.8486498, 2.459837</t>
+          <t>48.8520934, 2.4849953</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Pharmacie des Larris</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>supermarché</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2397,26 +2397,26 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>48.8543123</v>
+        <v>48.8556285</v>
       </c>
       <c r="E71" t="n">
-        <v>2.4864997</v>
+        <v>2.4777739</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>48.8543123, 2.4864997</t>
+          <t>48.8556285, 2.4777739</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Pharmacie du Marché</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>supermarché</t>
+          <t>pharmacie</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2425,40 +2425,432 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>48.8543623</v>
+        <v>48.8534714</v>
       </c>
       <c r="E72" t="n">
-        <v>2.4863951</v>
+        <v>2.4698085</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>48.8543623, 2.4863951</t>
+          <t>48.8534714, 2.4698085</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
+          <t>Pharmacie du village</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>pharmacie</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>48.8462203</v>
+      </c>
+      <c r="E73" t="n">
+        <v>2.4675405</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>48.8462203, 2.4675405</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Fontenay-sous-Bois Principal</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>poste</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>48.8490985</v>
+      </c>
+      <c r="E74" t="n">
+        <v>2.4755055</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>48.8490985, 2.4755055</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Fontenay-sous-Bois Rigollots</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>poste</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>48.848805</v>
+      </c>
+      <c r="E75" t="n">
+        <v>2.4579266</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>48.848805, 2.4579266</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Relais Postal</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>poste</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>48.853931</v>
+      </c>
+      <c r="E76" t="n">
+        <v>2.4695139</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>48.853931, 2.4695139</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Val-de-Fontenay</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>poste</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>48.853767</v>
+      </c>
+      <c r="E77" t="n">
+        <v>2.4876008</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>48.853767, 2.4876008</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Auchan</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>supermarché</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>48.8532361</v>
+      </c>
+      <c r="E78" t="n">
+        <v>2.4827546</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>48.8532361, 2.4827546</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Diagonal</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>supermarché</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>48.8559879</v>
+      </c>
+      <c r="E79" t="n">
+        <v>2.4784523</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>48.8559879, 2.4784523</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Hyper Casher</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>supermarché</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>48.8546063</v>
+      </c>
+      <c r="E80" t="n">
+        <v>2.4689527</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>48.8546063, 2.4689527</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Intermarché</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>supermarché</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>48.8495365</v>
+      </c>
+      <c r="E81" t="n">
+        <v>2.48986</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>48.8495365, 2.48986</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Lidl</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>supermarché</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>48.8485331</v>
+      </c>
+      <c r="E82" t="n">
+        <v>2.4886907</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>48.8485331, 2.4886907</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Monoprix</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>supermarché</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>48.8493017</v>
+      </c>
+      <c r="E83" t="n">
+        <v>2.458854</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>48.8493017, 2.458854</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Naturalia</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>supermarché</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>48.8486498</v>
+      </c>
+      <c r="E84" t="n">
+        <v>2.459837</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>48.8486498, 2.459837</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>supermarché</t>
         </is>
       </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>OpenStreetMap</t>
-        </is>
-      </c>
-      <c r="D73" t="n">
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>48.8543123</v>
+      </c>
+      <c r="E85" t="n">
+        <v>2.4864997</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>48.8543123, 2.4864997</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>supermarché</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>48.8543623</v>
+      </c>
+      <c r="E86" t="n">
+        <v>2.4863951</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>48.8543623, 2.4863951</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>supermarché</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>OpenStreetMap</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
         <v>48.8544087</v>
       </c>
-      <c r="E73" t="n">
+      <c r="E87" t="n">
         <v>2.4863051</v>
       </c>
-      <c r="F73" t="inlineStr">
+      <c r="F87" t="inlineStr">
         <is>
           <t>48.8544087, 2.4863051</t>
         </is>

</xml_diff>